<commit_message>
dados de tangará ajustado
</commit_message>
<xml_diff>
--- a/Tabela com codigos operativos.xlsx
+++ b/Tabela com codigos operativos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Engeselt\Documents\GitHub\ASPO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF6D4C1-9033-4700-9D97-44947FE30D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD614164-C45D-4977-8947-530E41EA4816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24497,27 +24497,15 @@
     <t>018TR04-EAE</t>
   </si>
   <si>
-    <t>SE TAN TR-04 13.8KV-EAE</t>
-  </si>
-  <si>
     <t>018TR04-EAR</t>
   </si>
   <si>
-    <t>SE TAN TR-04 13.8KV-EAR</t>
-  </si>
-  <si>
     <t>018TR04-ERE</t>
   </si>
   <si>
-    <t>SE TAN TR-04 13.8KV-ERE</t>
-  </si>
-  <si>
     <t>018TR04-ERR</t>
   </si>
   <si>
-    <t>SE TAN TR-04 13.8KV-ERR</t>
-  </si>
-  <si>
     <t>018TR01-EAE</t>
   </si>
   <si>
@@ -24545,27 +24533,15 @@
     <t>018TR03-EAE</t>
   </si>
   <si>
-    <t>SE TAN TR03 34.5KV-EAE</t>
-  </si>
-  <si>
     <t>018TR03-EAR</t>
   </si>
   <si>
-    <t>SE TAN TR03 34.5KV-EAR</t>
-  </si>
-  <si>
     <t>018TR03-ERE</t>
   </si>
   <si>
-    <t>SE TAN TR03 34.5KV-ERE</t>
-  </si>
-  <si>
     <t>018TR03-ERR</t>
   </si>
   <si>
-    <t>SE TAN TR03 34.5KV-ERR</t>
-  </si>
-  <si>
     <t>PCH FAXINAL I-EAE</t>
   </si>
   <si>
@@ -26424,6 +26400,30 @@
   </si>
   <si>
     <t>SE CN PARECIS TR-02 13.8KV-ERR</t>
+  </si>
+  <si>
+    <t>SE TAN TR04 34.5KV-EAE</t>
+  </si>
+  <si>
+    <t>SE TAN TR04 34.5KV-EAR</t>
+  </si>
+  <si>
+    <t>SE TAN TR04 34.5KV-ERE</t>
+  </si>
+  <si>
+    <t>SE TAN TR04 34.5KV-ERR</t>
+  </si>
+  <si>
+    <t>SE TAN TR-03 13.8KV-EAE</t>
+  </si>
+  <si>
+    <t>SE TAN TR-03 13.8KV-EAR</t>
+  </si>
+  <si>
+    <t>SE TAN TR-03 13.8KV-ERE</t>
+  </si>
+  <si>
+    <t>SE TAN TR-03 13.8KV-ERR</t>
   </si>
 </sst>
 </file>
@@ -57332,7 +57332,7 @@
         <v>7220</v>
       </c>
       <c r="B3758" t="s">
-        <v>8788</v>
+        <v>8780</v>
       </c>
     </row>
     <row r="3759" spans="1:2" x14ac:dyDescent="0.25">
@@ -57340,7 +57340,7 @@
         <v>7221</v>
       </c>
       <c r="B3759" t="s">
-        <v>8789</v>
+        <v>8781</v>
       </c>
     </row>
     <row r="3760" spans="1:2" x14ac:dyDescent="0.25">
@@ -57348,7 +57348,7 @@
         <v>7222</v>
       </c>
       <c r="B3760" t="s">
-        <v>8790</v>
+        <v>8782</v>
       </c>
     </row>
     <row r="3761" spans="1:2" x14ac:dyDescent="0.25">
@@ -57356,7 +57356,7 @@
         <v>7223</v>
       </c>
       <c r="B3761" t="s">
-        <v>8791</v>
+        <v>8783</v>
       </c>
     </row>
     <row r="3762" spans="1:2" x14ac:dyDescent="0.25">
@@ -57364,7 +57364,7 @@
         <v>7224</v>
       </c>
       <c r="B3762" t="s">
-        <v>8792</v>
+        <v>8784</v>
       </c>
     </row>
     <row r="3763" spans="1:2" x14ac:dyDescent="0.25">
@@ -57372,7 +57372,7 @@
         <v>7225</v>
       </c>
       <c r="B3763" t="s">
-        <v>8793</v>
+        <v>8785</v>
       </c>
     </row>
     <row r="3764" spans="1:2" x14ac:dyDescent="0.25">
@@ -57380,7 +57380,7 @@
         <v>7226</v>
       </c>
       <c r="B3764" t="s">
-        <v>8794</v>
+        <v>8786</v>
       </c>
     </row>
     <row r="3765" spans="1:2" x14ac:dyDescent="0.25">
@@ -57388,7 +57388,7 @@
         <v>7227</v>
       </c>
       <c r="B3765" t="s">
-        <v>8795</v>
+        <v>8787</v>
       </c>
     </row>
     <row r="3766" spans="1:2" x14ac:dyDescent="0.25">
@@ -61105,130 +61105,130 @@
     </row>
     <row r="4230" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4230" t="s">
-        <v>8152</v>
+        <v>8164</v>
       </c>
       <c r="B4230" t="s">
-        <v>8153</v>
+        <v>8792</v>
       </c>
     </row>
     <row r="4231" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4231" t="s">
-        <v>8154</v>
+        <v>8165</v>
       </c>
       <c r="B4231" t="s">
-        <v>8155</v>
+        <v>8793</v>
       </c>
     </row>
     <row r="4232" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4232" t="s">
-        <v>8156</v>
+        <v>8166</v>
       </c>
       <c r="B4232" t="s">
-        <v>8157</v>
+        <v>8794</v>
       </c>
     </row>
     <row r="4233" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4233" t="s">
-        <v>8158</v>
+        <v>8167</v>
       </c>
       <c r="B4233" t="s">
-        <v>8159</v>
+        <v>8795</v>
       </c>
     </row>
     <row r="4234" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4234" t="s">
-        <v>8160</v>
+        <v>8156</v>
       </c>
       <c r="B4234" t="s">
-        <v>8161</v>
+        <v>8157</v>
       </c>
     </row>
     <row r="4235" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4235" t="s">
-        <v>8162</v>
+        <v>8158</v>
       </c>
       <c r="B4235" t="s">
-        <v>8163</v>
+        <v>8159</v>
       </c>
     </row>
     <row r="4236" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4236" t="s">
-        <v>8164</v>
+        <v>8160</v>
       </c>
       <c r="B4236" t="s">
-        <v>8165</v>
+        <v>8161</v>
       </c>
     </row>
     <row r="4237" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4237" t="s">
-        <v>8166</v>
+        <v>8162</v>
       </c>
       <c r="B4237" t="s">
-        <v>8167</v>
+        <v>8163</v>
       </c>
     </row>
     <row r="4238" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4238" t="s">
-        <v>8168</v>
+        <v>8152</v>
       </c>
       <c r="B4238" t="s">
-        <v>8169</v>
+        <v>8788</v>
       </c>
     </row>
     <row r="4239" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4239" t="s">
-        <v>8170</v>
+        <v>8153</v>
       </c>
       <c r="B4239" t="s">
-        <v>8171</v>
+        <v>8789</v>
       </c>
     </row>
     <row r="4240" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4240" t="s">
-        <v>8172</v>
+        <v>8154</v>
       </c>
       <c r="B4240" t="s">
-        <v>8173</v>
+        <v>8790</v>
       </c>
     </row>
     <row r="4241" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4241" t="s">
-        <v>8174</v>
+        <v>8155</v>
       </c>
       <c r="B4241" t="s">
-        <v>8175</v>
+        <v>8791</v>
       </c>
     </row>
     <row r="4242" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4242" t="s">
-        <v>8176</v>
+        <v>8168</v>
       </c>
       <c r="B4242" t="s">
-        <v>8177</v>
+        <v>8169</v>
       </c>
     </row>
     <row r="4243" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4243" t="s">
-        <v>8178</v>
+        <v>8170</v>
       </c>
       <c r="B4243" t="s">
-        <v>8179</v>
+        <v>8171</v>
       </c>
     </row>
     <row r="4244" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4244" t="s">
-        <v>8180</v>
+        <v>8172</v>
       </c>
       <c r="B4244" t="s">
-        <v>8181</v>
+        <v>8173</v>
       </c>
     </row>
     <row r="4245" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4245" t="s">
-        <v>8182</v>
+        <v>8174</v>
       </c>
       <c r="B4245" t="s">
-        <v>8183</v>
+        <v>8175</v>
       </c>
     </row>
     <row r="4246" spans="1:2" x14ac:dyDescent="0.25">
@@ -61236,7 +61236,7 @@
         <v>154</v>
       </c>
       <c r="B4246" t="s">
-        <v>8184</v>
+        <v>8176</v>
       </c>
     </row>
     <row r="4247" spans="1:2" x14ac:dyDescent="0.25">
@@ -61244,7 +61244,7 @@
         <v>156</v>
       </c>
       <c r="B4247" t="s">
-        <v>8185</v>
+        <v>8177</v>
       </c>
     </row>
     <row r="4248" spans="1:2" x14ac:dyDescent="0.25">
@@ -61252,7 +61252,7 @@
         <v>158</v>
       </c>
       <c r="B4248" t="s">
-        <v>8186</v>
+        <v>8178</v>
       </c>
     </row>
     <row r="4249" spans="1:2" x14ac:dyDescent="0.25">
@@ -61260,359 +61260,359 @@
         <v>160</v>
       </c>
       <c r="B4249" t="s">
-        <v>8187</v>
+        <v>8179</v>
       </c>
     </row>
     <row r="4250" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4250" t="s">
-        <v>8188</v>
+        <v>8180</v>
       </c>
       <c r="B4250" t="s">
-        <v>8189</v>
+        <v>8181</v>
       </c>
     </row>
     <row r="4251" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4251" t="s">
-        <v>8190</v>
+        <v>8182</v>
       </c>
       <c r="B4251" t="s">
-        <v>8191</v>
+        <v>8183</v>
       </c>
     </row>
     <row r="4252" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4252" t="s">
-        <v>8192</v>
+        <v>8184</v>
       </c>
       <c r="B4252" t="s">
-        <v>8193</v>
+        <v>8185</v>
       </c>
     </row>
     <row r="4253" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4253" t="s">
-        <v>8194</v>
+        <v>8186</v>
       </c>
       <c r="B4253" t="s">
-        <v>8195</v>
+        <v>8187</v>
       </c>
     </row>
     <row r="4254" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4254" t="s">
-        <v>8196</v>
+        <v>8188</v>
       </c>
       <c r="B4254" t="s">
-        <v>8197</v>
+        <v>8189</v>
       </c>
     </row>
     <row r="4255" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4255" t="s">
-        <v>8198</v>
+        <v>8190</v>
       </c>
       <c r="B4255" t="s">
-        <v>8199</v>
+        <v>8191</v>
       </c>
     </row>
     <row r="4256" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4256" t="s">
-        <v>8200</v>
+        <v>8192</v>
       </c>
       <c r="B4256" t="s">
-        <v>8201</v>
+        <v>8193</v>
       </c>
     </row>
     <row r="4257" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4257" t="s">
-        <v>8202</v>
+        <v>8194</v>
       </c>
       <c r="B4257" t="s">
-        <v>8203</v>
+        <v>8195</v>
       </c>
     </row>
     <row r="4258" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4258" t="s">
-        <v>8204</v>
+        <v>8196</v>
       </c>
       <c r="B4258" t="s">
-        <v>8205</v>
+        <v>8197</v>
       </c>
     </row>
     <row r="4259" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4259" t="s">
-        <v>8206</v>
+        <v>8198</v>
       </c>
       <c r="B4259" t="s">
-        <v>8207</v>
+        <v>8199</v>
       </c>
     </row>
     <row r="4260" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4260" t="s">
-        <v>8208</v>
+        <v>8200</v>
       </c>
       <c r="B4260" t="s">
-        <v>8209</v>
+        <v>8201</v>
       </c>
     </row>
     <row r="4261" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4261" t="s">
-        <v>8210</v>
+        <v>8202</v>
       </c>
       <c r="B4261" t="s">
-        <v>8211</v>
+        <v>8203</v>
       </c>
     </row>
     <row r="4262" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4262" t="s">
-        <v>8212</v>
+        <v>8204</v>
       </c>
       <c r="B4262" t="s">
-        <v>8213</v>
+        <v>8205</v>
       </c>
     </row>
     <row r="4263" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4263" t="s">
-        <v>8214</v>
+        <v>8206</v>
       </c>
       <c r="B4263" t="s">
-        <v>8215</v>
+        <v>8207</v>
       </c>
     </row>
     <row r="4264" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4264" t="s">
-        <v>8216</v>
+        <v>8208</v>
       </c>
       <c r="B4264" t="s">
-        <v>8217</v>
+        <v>8209</v>
       </c>
     </row>
     <row r="4265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4265" t="s">
-        <v>8218</v>
+        <v>8210</v>
       </c>
       <c r="B4265" t="s">
-        <v>8219</v>
+        <v>8211</v>
       </c>
     </row>
     <row r="4266" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4266" t="s">
-        <v>8220</v>
+        <v>8212</v>
       </c>
       <c r="B4266" t="s">
-        <v>8221</v>
+        <v>8213</v>
       </c>
     </row>
     <row r="4267" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4267" t="s">
-        <v>8222</v>
+        <v>8214</v>
       </c>
       <c r="B4267" t="s">
-        <v>8223</v>
+        <v>8215</v>
       </c>
     </row>
     <row r="4268" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4268" t="s">
-        <v>8224</v>
+        <v>8216</v>
       </c>
       <c r="B4268" t="s">
-        <v>8225</v>
+        <v>8217</v>
       </c>
     </row>
     <row r="4269" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4269" t="s">
-        <v>8226</v>
+        <v>8218</v>
       </c>
       <c r="B4269" t="s">
-        <v>8227</v>
+        <v>8219</v>
       </c>
     </row>
     <row r="4270" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4270" t="s">
-        <v>8780</v>
+        <v>8772</v>
       </c>
       <c r="B4270" t="s">
-        <v>8784</v>
+        <v>8776</v>
       </c>
     </row>
     <row r="4271" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4271" t="s">
-        <v>8781</v>
+        <v>8773</v>
       </c>
       <c r="B4271" t="s">
-        <v>8784</v>
+        <v>8776</v>
       </c>
     </row>
     <row r="4272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4272" t="s">
-        <v>8782</v>
+        <v>8774</v>
       </c>
       <c r="B4272" t="s">
-        <v>8784</v>
+        <v>8776</v>
       </c>
     </row>
     <row r="4273" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4273" t="s">
-        <v>8783</v>
+        <v>8775</v>
       </c>
       <c r="B4273" t="s">
-        <v>8784</v>
+        <v>8776</v>
       </c>
     </row>
     <row r="4274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4274" t="s">
-        <v>8228</v>
+        <v>8220</v>
       </c>
       <c r="B4274" t="s">
-        <v>8229</v>
+        <v>8221</v>
       </c>
     </row>
     <row r="4275" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4275" t="s">
-        <v>8230</v>
+        <v>8222</v>
       </c>
       <c r="B4275" t="s">
-        <v>8231</v>
+        <v>8223</v>
       </c>
     </row>
     <row r="4276" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4276" t="s">
-        <v>8232</v>
+        <v>8224</v>
       </c>
       <c r="B4276" t="s">
-        <v>8233</v>
+        <v>8225</v>
       </c>
     </row>
     <row r="4277" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4277" t="s">
-        <v>8234</v>
+        <v>8226</v>
       </c>
       <c r="B4277" t="s">
-        <v>8235</v>
+        <v>8227</v>
       </c>
     </row>
     <row r="4278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4278" t="s">
-        <v>8236</v>
+        <v>8228</v>
       </c>
       <c r="B4278" t="s">
-        <v>8237</v>
+        <v>8229</v>
       </c>
     </row>
     <row r="4279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4279" t="s">
-        <v>8238</v>
+        <v>8230</v>
       </c>
       <c r="B4279" t="s">
-        <v>8239</v>
+        <v>8231</v>
       </c>
     </row>
     <row r="4280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4280" t="s">
-        <v>8240</v>
+        <v>8232</v>
       </c>
       <c r="B4280" t="s">
-        <v>8241</v>
+        <v>8233</v>
       </c>
     </row>
     <row r="4281" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4281" t="s">
-        <v>8242</v>
+        <v>8234</v>
       </c>
       <c r="B4281" t="s">
-        <v>8243</v>
+        <v>8235</v>
       </c>
     </row>
     <row r="4282" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4282" t="s">
-        <v>8244</v>
+        <v>8236</v>
       </c>
       <c r="B4282" t="s">
-        <v>8245</v>
+        <v>8237</v>
       </c>
     </row>
     <row r="4283" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4283" t="s">
-        <v>8246</v>
+        <v>8238</v>
       </c>
       <c r="B4283" t="s">
-        <v>8247</v>
+        <v>8239</v>
       </c>
     </row>
     <row r="4284" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4284" t="s">
-        <v>8248</v>
+        <v>8240</v>
       </c>
       <c r="B4284" t="s">
-        <v>8249</v>
+        <v>8241</v>
       </c>
     </row>
     <row r="4285" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4285" t="s">
-        <v>8250</v>
+        <v>8242</v>
       </c>
       <c r="B4285" t="s">
-        <v>8251</v>
+        <v>8243</v>
       </c>
     </row>
     <row r="4286" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4286" t="s">
-        <v>8252</v>
+        <v>8244</v>
       </c>
       <c r="B4286" t="s">
-        <v>8253</v>
+        <v>8245</v>
       </c>
     </row>
     <row r="4287" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4287" t="s">
-        <v>8254</v>
+        <v>8246</v>
       </c>
       <c r="B4287" t="s">
-        <v>8255</v>
+        <v>8247</v>
       </c>
     </row>
     <row r="4288" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4288" t="s">
-        <v>8256</v>
+        <v>8248</v>
       </c>
       <c r="B4288" t="s">
-        <v>8257</v>
+        <v>8249</v>
       </c>
     </row>
     <row r="4289" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4289" t="s">
-        <v>8258</v>
+        <v>8250</v>
       </c>
       <c r="B4289" t="s">
-        <v>8259</v>
+        <v>8251</v>
       </c>
     </row>
     <row r="4290" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4290" t="s">
-        <v>8260</v>
+        <v>8252</v>
       </c>
       <c r="B4290" t="s">
-        <v>8261</v>
+        <v>8253</v>
       </c>
     </row>
     <row r="4291" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4291" t="s">
-        <v>8262</v>
+        <v>8254</v>
       </c>
       <c r="B4291" t="s">
-        <v>8263</v>
+        <v>8255</v>
       </c>
     </row>
     <row r="4292" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4292" t="s">
-        <v>8264</v>
+        <v>8256</v>
       </c>
       <c r="B4292" t="s">
-        <v>8265</v>
+        <v>8257</v>
       </c>
     </row>
     <row r="4293" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4293" t="s">
-        <v>8266</v>
+        <v>8258</v>
       </c>
       <c r="B4293" t="s">
-        <v>8267</v>
+        <v>8259</v>
       </c>
     </row>
     <row r="4294" spans="1:2" x14ac:dyDescent="0.25">
@@ -61620,7 +61620,7 @@
         <v>#N/A</v>
       </c>
       <c r="B4294" t="s">
-        <v>8268</v>
+        <v>8260</v>
       </c>
     </row>
     <row r="4295" spans="1:2" x14ac:dyDescent="0.25">
@@ -61628,7 +61628,7 @@
         <v>#N/A</v>
       </c>
       <c r="B4295" t="s">
-        <v>8269</v>
+        <v>8261</v>
       </c>
     </row>
     <row r="4296" spans="1:2" x14ac:dyDescent="0.25">
@@ -61636,7 +61636,7 @@
         <v>#N/A</v>
       </c>
       <c r="B4296" t="s">
-        <v>8270</v>
+        <v>8262</v>
       </c>
     </row>
     <row r="4297" spans="1:2" x14ac:dyDescent="0.25">
@@ -61644,7 +61644,7 @@
         <v>#N/A</v>
       </c>
       <c r="B4297" t="s">
-        <v>8271</v>
+        <v>8263</v>
       </c>
     </row>
     <row r="4298" spans="1:2" x14ac:dyDescent="0.25">
@@ -61652,7 +61652,7 @@
         <v>#N/A</v>
       </c>
       <c r="B4298" t="s">
-        <v>8272</v>
+        <v>8264</v>
       </c>
     </row>
     <row r="4299" spans="1:2" x14ac:dyDescent="0.25">
@@ -61660,7 +61660,7 @@
         <v>#N/A</v>
       </c>
       <c r="B4299" t="s">
-        <v>8273</v>
+        <v>8265</v>
       </c>
     </row>
     <row r="4300" spans="1:2" x14ac:dyDescent="0.25">
@@ -61668,7 +61668,7 @@
         <v>#N/A</v>
       </c>
       <c r="B4300" t="s">
-        <v>8274</v>
+        <v>8266</v>
       </c>
     </row>
     <row r="4301" spans="1:2" x14ac:dyDescent="0.25">
@@ -61676,7 +61676,7 @@
         <v>#N/A</v>
       </c>
       <c r="B4301" t="s">
-        <v>8275</v>
+        <v>8267</v>
       </c>
     </row>
     <row r="4302" spans="1:2" x14ac:dyDescent="0.25">
@@ -61684,7 +61684,7 @@
         <v>154</v>
       </c>
       <c r="B4302" t="s">
-        <v>8276</v>
+        <v>8268</v>
       </c>
     </row>
     <row r="4303" spans="1:2" x14ac:dyDescent="0.25">
@@ -61692,7 +61692,7 @@
         <v>156</v>
       </c>
       <c r="B4303" t="s">
-        <v>8277</v>
+        <v>8269</v>
       </c>
     </row>
     <row r="4304" spans="1:2" x14ac:dyDescent="0.25">
@@ -61700,7 +61700,7 @@
         <v>158</v>
       </c>
       <c r="B4304" t="s">
-        <v>8278</v>
+        <v>8270</v>
       </c>
     </row>
     <row r="4305" spans="1:2" x14ac:dyDescent="0.25">
@@ -61708,7 +61708,7 @@
         <v>160</v>
       </c>
       <c r="B4305" t="s">
-        <v>8279</v>
+        <v>8271</v>
       </c>
     </row>
     <row r="4306" spans="1:2" x14ac:dyDescent="0.25">
@@ -61716,7 +61716,7 @@
         <v>154</v>
       </c>
       <c r="B4306" t="s">
-        <v>8280</v>
+        <v>8272</v>
       </c>
     </row>
     <row r="4307" spans="1:2" x14ac:dyDescent="0.25">
@@ -61724,7 +61724,7 @@
         <v>156</v>
       </c>
       <c r="B4307" t="s">
-        <v>8281</v>
+        <v>8273</v>
       </c>
     </row>
     <row r="4308" spans="1:2" x14ac:dyDescent="0.25">
@@ -61732,7 +61732,7 @@
         <v>158</v>
       </c>
       <c r="B4308" t="s">
-        <v>8282</v>
+        <v>8274</v>
       </c>
     </row>
     <row r="4309" spans="1:2" x14ac:dyDescent="0.25">
@@ -61740,7 +61740,7 @@
         <v>160</v>
       </c>
       <c r="B4309" t="s">
-        <v>8283</v>
+        <v>8275</v>
       </c>
     </row>
     <row r="4310" spans="1:2" x14ac:dyDescent="0.25">
@@ -61748,7 +61748,7 @@
         <v>154</v>
       </c>
       <c r="B4310" t="s">
-        <v>8284</v>
+        <v>8276</v>
       </c>
     </row>
     <row r="4311" spans="1:2" x14ac:dyDescent="0.25">
@@ -61756,7 +61756,7 @@
         <v>156</v>
       </c>
       <c r="B4311" t="s">
-        <v>8285</v>
+        <v>8277</v>
       </c>
     </row>
     <row r="4312" spans="1:2" x14ac:dyDescent="0.25">
@@ -61764,7 +61764,7 @@
         <v>158</v>
       </c>
       <c r="B4312" t="s">
-        <v>8286</v>
+        <v>8278</v>
       </c>
     </row>
     <row r="4313" spans="1:2" x14ac:dyDescent="0.25">
@@ -61772,7 +61772,7 @@
         <v>160</v>
       </c>
       <c r="B4313" t="s">
-        <v>8287</v>
+        <v>8279</v>
       </c>
     </row>
     <row r="4314" spans="1:2" x14ac:dyDescent="0.25">
@@ -61780,7 +61780,7 @@
         <v>154</v>
       </c>
       <c r="B4314" t="s">
-        <v>8288</v>
+        <v>8280</v>
       </c>
     </row>
     <row r="4315" spans="1:2" x14ac:dyDescent="0.25">
@@ -61788,7 +61788,7 @@
         <v>156</v>
       </c>
       <c r="B4315" t="s">
-        <v>8289</v>
+        <v>8281</v>
       </c>
     </row>
     <row r="4316" spans="1:2" x14ac:dyDescent="0.25">
@@ -61796,7 +61796,7 @@
         <v>158</v>
       </c>
       <c r="B4316" t="s">
-        <v>8290</v>
+        <v>8282</v>
       </c>
     </row>
     <row r="4317" spans="1:2" x14ac:dyDescent="0.25">
@@ -61804,7 +61804,7 @@
         <v>160</v>
       </c>
       <c r="B4317" t="s">
-        <v>8291</v>
+        <v>8283</v>
       </c>
     </row>
     <row r="4318" spans="1:2" x14ac:dyDescent="0.25">
@@ -61812,7 +61812,7 @@
         <v>154</v>
       </c>
       <c r="B4318" t="s">
-        <v>8292</v>
+        <v>8284</v>
       </c>
     </row>
     <row r="4319" spans="1:2" x14ac:dyDescent="0.25">
@@ -61820,7 +61820,7 @@
         <v>156</v>
       </c>
       <c r="B4319" t="s">
-        <v>8293</v>
+        <v>8285</v>
       </c>
     </row>
     <row r="4320" spans="1:2" x14ac:dyDescent="0.25">
@@ -61828,7 +61828,7 @@
         <v>158</v>
       </c>
       <c r="B4320" t="s">
-        <v>8294</v>
+        <v>8286</v>
       </c>
     </row>
     <row r="4321" spans="1:2" x14ac:dyDescent="0.25">
@@ -61836,7 +61836,7 @@
         <v>160</v>
       </c>
       <c r="B4321" t="s">
-        <v>8295</v>
+        <v>8287</v>
       </c>
     </row>
     <row r="4322" spans="1:2" x14ac:dyDescent="0.25">
@@ -61844,7 +61844,7 @@
         <v>154</v>
       </c>
       <c r="B4322" t="s">
-        <v>8296</v>
+        <v>8288</v>
       </c>
     </row>
     <row r="4323" spans="1:2" x14ac:dyDescent="0.25">
@@ -61852,7 +61852,7 @@
         <v>156</v>
       </c>
       <c r="B4323" t="s">
-        <v>8297</v>
+        <v>8289</v>
       </c>
     </row>
     <row r="4324" spans="1:2" x14ac:dyDescent="0.25">
@@ -61860,7 +61860,7 @@
         <v>158</v>
       </c>
       <c r="B4324" t="s">
-        <v>8298</v>
+        <v>8290</v>
       </c>
     </row>
     <row r="4325" spans="1:2" x14ac:dyDescent="0.25">
@@ -61868,1383 +61868,1383 @@
         <v>160</v>
       </c>
       <c r="B4325" t="s">
-        <v>8299</v>
+        <v>8291</v>
       </c>
     </row>
     <row r="4326" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4326" t="s">
-        <v>8300</v>
+        <v>8292</v>
       </c>
       <c r="B4326" t="s">
-        <v>8301</v>
+        <v>8293</v>
       </c>
     </row>
     <row r="4327" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4327" t="s">
-        <v>8302</v>
+        <v>8294</v>
       </c>
       <c r="B4327" t="s">
-        <v>8303</v>
+        <v>8295</v>
       </c>
     </row>
     <row r="4328" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4328" t="s">
-        <v>8304</v>
+        <v>8296</v>
       </c>
       <c r="B4328" t="s">
-        <v>8305</v>
+        <v>8297</v>
       </c>
     </row>
     <row r="4329" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4329" t="s">
-        <v>8306</v>
+        <v>8298</v>
       </c>
       <c r="B4329" t="s">
-        <v>8307</v>
+        <v>8299</v>
       </c>
     </row>
     <row r="4330" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4330" t="s">
-        <v>8308</v>
+        <v>8300</v>
       </c>
       <c r="B4330" t="s">
-        <v>8309</v>
+        <v>8301</v>
       </c>
     </row>
     <row r="4331" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4331" t="s">
-        <v>8310</v>
+        <v>8302</v>
       </c>
       <c r="B4331" t="s">
-        <v>8311</v>
+        <v>8303</v>
       </c>
     </row>
     <row r="4332" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4332" t="s">
-        <v>8312</v>
+        <v>8304</v>
       </c>
       <c r="B4332" t="s">
-        <v>8313</v>
+        <v>8305</v>
       </c>
     </row>
     <row r="4333" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4333" t="s">
-        <v>8314</v>
+        <v>8306</v>
       </c>
       <c r="B4333" t="s">
-        <v>8315</v>
+        <v>8307</v>
       </c>
     </row>
     <row r="4334" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4334" t="s">
-        <v>8316</v>
+        <v>8308</v>
       </c>
       <c r="B4334" t="s">
-        <v>8317</v>
+        <v>8309</v>
       </c>
     </row>
     <row r="4335" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4335" t="s">
-        <v>8318</v>
+        <v>8310</v>
       </c>
       <c r="B4335" t="s">
-        <v>8319</v>
+        <v>8311</v>
       </c>
     </row>
     <row r="4336" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4336" t="s">
-        <v>8320</v>
+        <v>8312</v>
       </c>
       <c r="B4336" t="s">
-        <v>8321</v>
+        <v>8313</v>
       </c>
     </row>
     <row r="4337" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4337" t="s">
-        <v>8322</v>
+        <v>8314</v>
       </c>
       <c r="B4337" t="s">
-        <v>8323</v>
+        <v>8315</v>
       </c>
     </row>
     <row r="4338" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4338" t="s">
-        <v>8324</v>
+        <v>8316</v>
       </c>
       <c r="B4338" t="s">
-        <v>8325</v>
+        <v>8317</v>
       </c>
     </row>
     <row r="4339" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4339" t="s">
-        <v>8326</v>
+        <v>8318</v>
       </c>
       <c r="B4339" t="s">
-        <v>8327</v>
+        <v>8319</v>
       </c>
     </row>
     <row r="4340" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4340" t="s">
-        <v>8328</v>
+        <v>8320</v>
       </c>
       <c r="B4340" t="s">
-        <v>8329</v>
+        <v>8321</v>
       </c>
     </row>
     <row r="4341" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4341" t="s">
-        <v>8330</v>
+        <v>8322</v>
       </c>
       <c r="B4341" t="s">
-        <v>8331</v>
+        <v>8323</v>
       </c>
     </row>
     <row r="4342" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4342" t="s">
-        <v>8332</v>
+        <v>8324</v>
       </c>
       <c r="B4342" t="s">
-        <v>8333</v>
+        <v>8325</v>
       </c>
     </row>
     <row r="4343" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4343" t="s">
-        <v>8334</v>
+        <v>8326</v>
       </c>
       <c r="B4343" t="s">
-        <v>8335</v>
+        <v>8327</v>
       </c>
     </row>
     <row r="4344" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4344" t="s">
-        <v>8336</v>
+        <v>8328</v>
       </c>
       <c r="B4344" t="s">
-        <v>8337</v>
+        <v>8329</v>
       </c>
     </row>
     <row r="4345" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4345" t="s">
-        <v>8338</v>
+        <v>8330</v>
       </c>
       <c r="B4345" t="s">
-        <v>8339</v>
+        <v>8331</v>
       </c>
     </row>
     <row r="4346" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4346" t="s">
-        <v>8340</v>
+        <v>8332</v>
       </c>
       <c r="B4346" t="s">
-        <v>8341</v>
+        <v>8333</v>
       </c>
     </row>
     <row r="4347" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4347" t="s">
-        <v>8342</v>
+        <v>8334</v>
       </c>
       <c r="B4347" t="s">
-        <v>8343</v>
+        <v>8335</v>
       </c>
     </row>
     <row r="4348" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4348" t="s">
-        <v>8344</v>
+        <v>8336</v>
       </c>
       <c r="B4348" t="s">
-        <v>8345</v>
+        <v>8337</v>
       </c>
     </row>
     <row r="4349" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4349" t="s">
-        <v>8346</v>
+        <v>8338</v>
       </c>
       <c r="B4349" t="s">
-        <v>8347</v>
+        <v>8339</v>
       </c>
     </row>
     <row r="4350" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4350" t="s">
-        <v>8348</v>
+        <v>8340</v>
       </c>
       <c r="B4350" t="s">
-        <v>8349</v>
+        <v>8341</v>
       </c>
     </row>
     <row r="4351" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4351" t="s">
-        <v>8350</v>
+        <v>8342</v>
       </c>
       <c r="B4351" t="s">
-        <v>8351</v>
+        <v>8343</v>
       </c>
     </row>
     <row r="4352" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4352" t="s">
-        <v>8352</v>
+        <v>8344</v>
       </c>
       <c r="B4352" t="s">
-        <v>8353</v>
+        <v>8345</v>
       </c>
     </row>
     <row r="4353" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4353" t="s">
-        <v>8354</v>
+        <v>8346</v>
       </c>
       <c r="B4353" t="s">
-        <v>8355</v>
+        <v>8347</v>
       </c>
     </row>
     <row r="4354" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4354" t="s">
-        <v>8356</v>
+        <v>8348</v>
       </c>
       <c r="B4354" t="s">
-        <v>8357</v>
+        <v>8349</v>
       </c>
     </row>
     <row r="4355" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4355" t="s">
-        <v>8358</v>
+        <v>8350</v>
       </c>
       <c r="B4355" t="s">
-        <v>8359</v>
+        <v>8351</v>
       </c>
     </row>
     <row r="4356" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4356" t="s">
-        <v>8360</v>
+        <v>8352</v>
       </c>
       <c r="B4356" t="s">
-        <v>8361</v>
+        <v>8353</v>
       </c>
     </row>
     <row r="4357" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4357" t="s">
-        <v>8362</v>
+        <v>8354</v>
       </c>
       <c r="B4357" t="s">
-        <v>8363</v>
+        <v>8355</v>
       </c>
     </row>
     <row r="4358" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4358" t="s">
-        <v>8364</v>
+        <v>8356</v>
       </c>
       <c r="B4358" t="s">
-        <v>8365</v>
+        <v>8357</v>
       </c>
     </row>
     <row r="4359" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4359" t="s">
-        <v>8366</v>
+        <v>8358</v>
       </c>
       <c r="B4359" t="s">
-        <v>8367</v>
+        <v>8359</v>
       </c>
     </row>
     <row r="4360" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4360" t="s">
-        <v>8368</v>
+        <v>8360</v>
       </c>
       <c r="B4360" t="s">
-        <v>8369</v>
+        <v>8361</v>
       </c>
     </row>
     <row r="4361" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4361" t="s">
-        <v>8370</v>
+        <v>8362</v>
       </c>
       <c r="B4361" t="s">
-        <v>8371</v>
+        <v>8363</v>
       </c>
     </row>
     <row r="4362" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4362" t="s">
-        <v>8372</v>
+        <v>8364</v>
       </c>
       <c r="B4362" t="s">
-        <v>8373</v>
+        <v>8365</v>
       </c>
     </row>
     <row r="4363" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4363" t="s">
-        <v>8374</v>
+        <v>8366</v>
       </c>
       <c r="B4363" t="s">
-        <v>8375</v>
+        <v>8367</v>
       </c>
     </row>
     <row r="4364" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4364" t="s">
-        <v>8376</v>
+        <v>8368</v>
       </c>
       <c r="B4364" t="s">
-        <v>8377</v>
+        <v>8369</v>
       </c>
     </row>
     <row r="4365" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4365" t="s">
-        <v>8378</v>
+        <v>8370</v>
       </c>
       <c r="B4365" t="s">
-        <v>8379</v>
+        <v>8371</v>
       </c>
     </row>
     <row r="4366" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4366" t="s">
-        <v>8380</v>
+        <v>8372</v>
       </c>
       <c r="B4366" t="s">
-        <v>8381</v>
+        <v>8373</v>
       </c>
     </row>
     <row r="4367" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4367" t="s">
-        <v>8382</v>
+        <v>8374</v>
       </c>
       <c r="B4367" t="s">
-        <v>8383</v>
+        <v>8375</v>
       </c>
     </row>
     <row r="4368" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4368" t="s">
-        <v>8384</v>
+        <v>8376</v>
       </c>
       <c r="B4368" t="s">
-        <v>8385</v>
+        <v>8377</v>
       </c>
     </row>
     <row r="4369" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4369" t="s">
-        <v>8386</v>
+        <v>8378</v>
       </c>
       <c r="B4369" t="s">
-        <v>8387</v>
+        <v>8379</v>
       </c>
     </row>
     <row r="4370" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4370" t="s">
-        <v>8388</v>
+        <v>8380</v>
       </c>
       <c r="B4370" t="s">
-        <v>8389</v>
+        <v>8381</v>
       </c>
     </row>
     <row r="4371" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4371" t="s">
-        <v>8390</v>
+        <v>8382</v>
       </c>
       <c r="B4371" t="s">
-        <v>8391</v>
+        <v>8383</v>
       </c>
     </row>
     <row r="4372" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4372" t="s">
-        <v>8392</v>
+        <v>8384</v>
       </c>
       <c r="B4372" t="s">
-        <v>8393</v>
+        <v>8385</v>
       </c>
     </row>
     <row r="4373" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4373" t="s">
-        <v>8394</v>
+        <v>8386</v>
       </c>
       <c r="B4373" t="s">
-        <v>8395</v>
+        <v>8387</v>
       </c>
     </row>
     <row r="4374" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4374" t="s">
-        <v>8396</v>
+        <v>8388</v>
       </c>
       <c r="B4374" t="s">
-        <v>8397</v>
+        <v>8389</v>
       </c>
     </row>
     <row r="4375" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4375" t="s">
-        <v>8398</v>
+        <v>8390</v>
       </c>
       <c r="B4375" t="s">
-        <v>8399</v>
+        <v>8391</v>
       </c>
     </row>
     <row r="4376" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4376" t="s">
-        <v>8400</v>
+        <v>8392</v>
       </c>
       <c r="B4376" t="s">
-        <v>8401</v>
+        <v>8393</v>
       </c>
     </row>
     <row r="4377" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4377" t="s">
-        <v>8402</v>
+        <v>8394</v>
       </c>
       <c r="B4377" t="s">
-        <v>8403</v>
+        <v>8395</v>
       </c>
     </row>
     <row r="4378" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4378" t="s">
-        <v>8404</v>
+        <v>8396</v>
       </c>
       <c r="B4378" t="s">
-        <v>8405</v>
+        <v>8397</v>
       </c>
     </row>
     <row r="4379" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4379" t="s">
-        <v>8406</v>
+        <v>8398</v>
       </c>
       <c r="B4379" t="s">
-        <v>8407</v>
+        <v>8399</v>
       </c>
     </row>
     <row r="4380" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4380" t="s">
-        <v>8408</v>
+        <v>8400</v>
       </c>
       <c r="B4380" t="s">
-        <v>8409</v>
+        <v>8401</v>
       </c>
     </row>
     <row r="4381" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4381" t="s">
-        <v>8410</v>
+        <v>8402</v>
       </c>
       <c r="B4381" t="s">
-        <v>8411</v>
+        <v>8403</v>
       </c>
     </row>
     <row r="4382" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4382" t="s">
-        <v>8412</v>
+        <v>8404</v>
       </c>
       <c r="B4382" t="s">
-        <v>8413</v>
+        <v>8405</v>
       </c>
     </row>
     <row r="4383" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4383" t="s">
-        <v>8414</v>
+        <v>8406</v>
       </c>
       <c r="B4383" t="s">
-        <v>8415</v>
+        <v>8407</v>
       </c>
     </row>
     <row r="4384" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4384" t="s">
-        <v>8416</v>
+        <v>8408</v>
       </c>
       <c r="B4384" t="s">
-        <v>8417</v>
+        <v>8409</v>
       </c>
     </row>
     <row r="4385" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4385" t="s">
-        <v>8418</v>
+        <v>8410</v>
       </c>
       <c r="B4385" t="s">
-        <v>8419</v>
+        <v>8411</v>
       </c>
     </row>
     <row r="4386" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4386" t="s">
-        <v>8420</v>
+        <v>8412</v>
       </c>
       <c r="B4386" t="s">
-        <v>8421</v>
+        <v>8413</v>
       </c>
     </row>
     <row r="4387" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4387" t="s">
-        <v>8422</v>
+        <v>8414</v>
       </c>
       <c r="B4387" t="s">
-        <v>8423</v>
+        <v>8415</v>
       </c>
     </row>
     <row r="4388" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4388" t="s">
-        <v>8424</v>
+        <v>8416</v>
       </c>
       <c r="B4388" t="s">
-        <v>8425</v>
+        <v>8417</v>
       </c>
     </row>
     <row r="4389" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4389" t="s">
-        <v>8426</v>
+        <v>8418</v>
       </c>
       <c r="B4389" t="s">
-        <v>8427</v>
+        <v>8419</v>
       </c>
     </row>
     <row r="4390" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4390" t="s">
-        <v>8428</v>
+        <v>8420</v>
       </c>
       <c r="B4390" t="s">
-        <v>8429</v>
+        <v>8421</v>
       </c>
     </row>
     <row r="4391" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4391" t="s">
-        <v>8430</v>
+        <v>8422</v>
       </c>
       <c r="B4391" t="s">
-        <v>8431</v>
+        <v>8423</v>
       </c>
     </row>
     <row r="4392" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4392" t="s">
-        <v>8432</v>
+        <v>8424</v>
       </c>
       <c r="B4392" t="s">
-        <v>8433</v>
+        <v>8425</v>
       </c>
     </row>
     <row r="4393" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4393" t="s">
-        <v>8434</v>
+        <v>8426</v>
       </c>
       <c r="B4393" t="s">
-        <v>8435</v>
+        <v>8427</v>
       </c>
     </row>
     <row r="4394" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4394" t="s">
-        <v>8436</v>
+        <v>8428</v>
       </c>
       <c r="B4394" t="s">
-        <v>8437</v>
+        <v>8429</v>
       </c>
     </row>
     <row r="4395" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4395" t="s">
-        <v>8438</v>
+        <v>8430</v>
       </c>
       <c r="B4395" t="s">
-        <v>8439</v>
+        <v>8431</v>
       </c>
     </row>
     <row r="4396" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4396" t="s">
-        <v>8440</v>
+        <v>8432</v>
       </c>
       <c r="B4396" t="s">
-        <v>8441</v>
+        <v>8433</v>
       </c>
     </row>
     <row r="4397" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4397" t="s">
-        <v>8442</v>
+        <v>8434</v>
       </c>
       <c r="B4397" t="s">
-        <v>8443</v>
+        <v>8435</v>
       </c>
     </row>
     <row r="4398" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4398" t="s">
-        <v>8444</v>
+        <v>8436</v>
       </c>
       <c r="B4398" t="s">
-        <v>8445</v>
+        <v>8437</v>
       </c>
     </row>
     <row r="4399" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4399" t="s">
-        <v>8446</v>
+        <v>8438</v>
       </c>
       <c r="B4399" t="s">
-        <v>8447</v>
+        <v>8439</v>
       </c>
     </row>
     <row r="4400" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4400" t="s">
-        <v>8448</v>
+        <v>8440</v>
       </c>
       <c r="B4400" t="s">
-        <v>8449</v>
+        <v>8441</v>
       </c>
     </row>
     <row r="4401" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4401" t="s">
-        <v>8450</v>
+        <v>8442</v>
       </c>
       <c r="B4401" t="s">
-        <v>8451</v>
+        <v>8443</v>
       </c>
     </row>
     <row r="4402" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4402" t="s">
-        <v>8452</v>
+        <v>8444</v>
       </c>
       <c r="B4402" t="s">
-        <v>8301</v>
+        <v>8293</v>
       </c>
     </row>
     <row r="4403" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4403" t="s">
-        <v>8453</v>
+        <v>8445</v>
       </c>
       <c r="B4403" t="s">
-        <v>8303</v>
+        <v>8295</v>
       </c>
     </row>
     <row r="4404" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4404" t="s">
-        <v>8454</v>
+        <v>8446</v>
       </c>
       <c r="B4404" t="s">
-        <v>8305</v>
+        <v>8297</v>
       </c>
     </row>
     <row r="4405" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4405" t="s">
-        <v>8455</v>
+        <v>8447</v>
       </c>
       <c r="B4405" t="s">
-        <v>8307</v>
+        <v>8299</v>
       </c>
     </row>
     <row r="4406" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4406" t="s">
-        <v>8456</v>
+        <v>8448</v>
       </c>
       <c r="B4406" t="s">
-        <v>8457</v>
+        <v>8449</v>
       </c>
     </row>
     <row r="4407" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4407" t="s">
-        <v>8458</v>
+        <v>8450</v>
       </c>
       <c r="B4407" t="s">
-        <v>8459</v>
+        <v>8451</v>
       </c>
     </row>
     <row r="4408" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4408" t="s">
-        <v>8460</v>
+        <v>8452</v>
       </c>
       <c r="B4408" t="s">
-        <v>8461</v>
+        <v>8453</v>
       </c>
     </row>
     <row r="4409" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4409" t="s">
-        <v>8462</v>
+        <v>8454</v>
       </c>
       <c r="B4409" t="s">
-        <v>8463</v>
+        <v>8455</v>
       </c>
     </row>
     <row r="4410" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4410" t="s">
-        <v>8464</v>
+        <v>8456</v>
       </c>
       <c r="B4410" t="s">
-        <v>8465</v>
+        <v>8457</v>
       </c>
     </row>
     <row r="4411" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4411" t="s">
-        <v>8466</v>
+        <v>8458</v>
       </c>
       <c r="B4411" t="s">
-        <v>8467</v>
+        <v>8459</v>
       </c>
     </row>
     <row r="4412" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4412" t="s">
-        <v>8468</v>
+        <v>8460</v>
       </c>
       <c r="B4412" t="s">
-        <v>8469</v>
+        <v>8461</v>
       </c>
     </row>
     <row r="4413" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4413" t="s">
-        <v>8470</v>
+        <v>8462</v>
       </c>
       <c r="B4413" t="s">
-        <v>8471</v>
+        <v>8463</v>
       </c>
     </row>
     <row r="4414" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4414" t="s">
-        <v>8472</v>
+        <v>8464</v>
       </c>
       <c r="B4414" t="s">
-        <v>8473</v>
+        <v>8465</v>
       </c>
     </row>
     <row r="4415" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4415" t="s">
-        <v>8474</v>
+        <v>8466</v>
       </c>
       <c r="B4415" t="s">
-        <v>8475</v>
+        <v>8467</v>
       </c>
     </row>
     <row r="4416" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4416" t="s">
-        <v>8476</v>
+        <v>8468</v>
       </c>
       <c r="B4416" t="s">
-        <v>8477</v>
+        <v>8469</v>
       </c>
     </row>
     <row r="4417" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4417" t="s">
-        <v>8478</v>
+        <v>8470</v>
       </c>
       <c r="B4417" t="s">
-        <v>8479</v>
+        <v>8471</v>
       </c>
     </row>
     <row r="4418" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4418" t="s">
-        <v>8480</v>
+        <v>8472</v>
       </c>
       <c r="B4418" t="s">
-        <v>8481</v>
+        <v>8473</v>
       </c>
     </row>
     <row r="4419" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4419" t="s">
-        <v>8482</v>
+        <v>8474</v>
       </c>
       <c r="B4419" t="s">
-        <v>8483</v>
+        <v>8475</v>
       </c>
     </row>
     <row r="4420" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4420" t="s">
-        <v>8484</v>
+        <v>8476</v>
       </c>
       <c r="B4420" t="s">
-        <v>8485</v>
+        <v>8477</v>
       </c>
     </row>
     <row r="4421" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4421" t="s">
-        <v>8486</v>
+        <v>8478</v>
       </c>
       <c r="B4421" t="s">
-        <v>8487</v>
+        <v>8479</v>
       </c>
     </row>
     <row r="4422" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4422" t="s">
-        <v>8488</v>
+        <v>8480</v>
       </c>
       <c r="B4422" t="s">
-        <v>8489</v>
+        <v>8481</v>
       </c>
     </row>
     <row r="4423" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4423" t="s">
-        <v>8490</v>
+        <v>8482</v>
       </c>
       <c r="B4423" t="s">
-        <v>8491</v>
+        <v>8483</v>
       </c>
     </row>
     <row r="4424" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4424" t="s">
-        <v>8492</v>
+        <v>8484</v>
       </c>
       <c r="B4424" t="s">
-        <v>8493</v>
+        <v>8485</v>
       </c>
     </row>
     <row r="4425" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4425" t="s">
-        <v>8494</v>
+        <v>8486</v>
       </c>
       <c r="B4425" t="s">
-        <v>8495</v>
+        <v>8487</v>
       </c>
     </row>
     <row r="4426" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4426" t="s">
-        <v>8496</v>
+        <v>8488</v>
       </c>
       <c r="B4426" t="s">
-        <v>8497</v>
+        <v>8489</v>
       </c>
     </row>
     <row r="4427" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4427" t="s">
-        <v>8498</v>
+        <v>8490</v>
       </c>
       <c r="B4427" t="s">
-        <v>8499</v>
+        <v>8491</v>
       </c>
     </row>
     <row r="4428" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4428" t="s">
-        <v>8500</v>
+        <v>8492</v>
       </c>
       <c r="B4428" t="s">
-        <v>8501</v>
+        <v>8493</v>
       </c>
     </row>
     <row r="4429" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4429" t="s">
-        <v>8502</v>
+        <v>8494</v>
       </c>
       <c r="B4429" t="s">
-        <v>8503</v>
+        <v>8495</v>
       </c>
     </row>
     <row r="4430" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4430" t="s">
-        <v>8504</v>
+        <v>8496</v>
       </c>
       <c r="B4430" t="s">
-        <v>8505</v>
+        <v>8497</v>
       </c>
     </row>
     <row r="4431" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4431" t="s">
-        <v>8506</v>
+        <v>8498</v>
       </c>
       <c r="B4431" t="s">
-        <v>8507</v>
+        <v>8499</v>
       </c>
     </row>
     <row r="4432" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4432" t="s">
-        <v>8508</v>
+        <v>8500</v>
       </c>
       <c r="B4432" t="s">
-        <v>8509</v>
+        <v>8501</v>
       </c>
     </row>
     <row r="4433" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4433" t="s">
-        <v>8510</v>
+        <v>8502</v>
       </c>
       <c r="B4433" t="s">
-        <v>8511</v>
+        <v>8503</v>
       </c>
     </row>
     <row r="4434" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4434" t="s">
-        <v>8512</v>
+        <v>8504</v>
       </c>
       <c r="B4434" t="s">
-        <v>8513</v>
+        <v>8505</v>
       </c>
     </row>
     <row r="4435" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4435" t="s">
-        <v>8514</v>
+        <v>8506</v>
       </c>
       <c r="B4435" t="s">
-        <v>8515</v>
+        <v>8507</v>
       </c>
     </row>
     <row r="4436" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4436" t="s">
-        <v>8516</v>
+        <v>8508</v>
       </c>
       <c r="B4436" t="s">
-        <v>8517</v>
+        <v>8509</v>
       </c>
     </row>
     <row r="4437" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4437" t="s">
-        <v>8518</v>
+        <v>8510</v>
       </c>
       <c r="B4437" t="s">
-        <v>8519</v>
+        <v>8511</v>
       </c>
     </row>
     <row r="4438" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4438" t="s">
-        <v>8520</v>
+        <v>8512</v>
       </c>
       <c r="B4438" t="s">
-        <v>8521</v>
+        <v>8513</v>
       </c>
     </row>
     <row r="4439" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4439" t="s">
-        <v>8522</v>
+        <v>8514</v>
       </c>
       <c r="B4439" t="s">
-        <v>8523</v>
+        <v>8515</v>
       </c>
     </row>
     <row r="4440" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4440" t="s">
-        <v>8524</v>
+        <v>8516</v>
       </c>
       <c r="B4440" t="s">
-        <v>8525</v>
+        <v>8517</v>
       </c>
     </row>
     <row r="4441" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4441" t="s">
-        <v>8526</v>
+        <v>8518</v>
       </c>
       <c r="B4441" t="s">
-        <v>8527</v>
+        <v>8519</v>
       </c>
     </row>
     <row r="4442" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4442" t="s">
-        <v>8528</v>
+        <v>8520</v>
       </c>
       <c r="B4442" t="s">
-        <v>8529</v>
+        <v>8521</v>
       </c>
     </row>
     <row r="4443" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4443" t="s">
-        <v>8530</v>
+        <v>8522</v>
       </c>
       <c r="B4443" t="s">
-        <v>8531</v>
+        <v>8523</v>
       </c>
     </row>
     <row r="4444" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4444" t="s">
-        <v>8532</v>
+        <v>8524</v>
       </c>
       <c r="B4444" t="s">
-        <v>8533</v>
+        <v>8525</v>
       </c>
     </row>
     <row r="4445" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4445" t="s">
-        <v>8534</v>
+        <v>8526</v>
       </c>
       <c r="B4445" t="s">
-        <v>8535</v>
+        <v>8527</v>
       </c>
     </row>
     <row r="4446" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4446" t="s">
-        <v>8536</v>
+        <v>8528</v>
       </c>
       <c r="B4446" t="s">
-        <v>8537</v>
+        <v>8529</v>
       </c>
     </row>
     <row r="4447" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4447" t="s">
-        <v>8538</v>
+        <v>8530</v>
       </c>
       <c r="B4447" t="s">
-        <v>8539</v>
+        <v>8531</v>
       </c>
     </row>
     <row r="4448" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4448" t="s">
-        <v>8540</v>
+        <v>8532</v>
       </c>
       <c r="B4448" t="s">
-        <v>8541</v>
+        <v>8533</v>
       </c>
     </row>
     <row r="4449" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4449" t="s">
-        <v>8542</v>
+        <v>8534</v>
       </c>
       <c r="B4449" t="s">
-        <v>8543</v>
+        <v>8535</v>
       </c>
     </row>
     <row r="4450" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4450" t="s">
-        <v>8544</v>
+        <v>8536</v>
       </c>
       <c r="B4450" t="s">
-        <v>8545</v>
+        <v>8537</v>
       </c>
     </row>
     <row r="4451" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4451" t="s">
-        <v>8546</v>
+        <v>8538</v>
       </c>
       <c r="B4451" t="s">
-        <v>8547</v>
+        <v>8539</v>
       </c>
     </row>
     <row r="4452" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4452" t="s">
-        <v>8548</v>
+        <v>8540</v>
       </c>
       <c r="B4452" t="s">
-        <v>8549</v>
+        <v>8541</v>
       </c>
     </row>
     <row r="4453" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4453" t="s">
-        <v>8550</v>
+        <v>8542</v>
       </c>
       <c r="B4453" t="s">
-        <v>8551</v>
+        <v>8543</v>
       </c>
     </row>
     <row r="4454" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4454" t="s">
-        <v>8552</v>
+        <v>8544</v>
       </c>
       <c r="B4454" t="s">
-        <v>8553</v>
+        <v>8545</v>
       </c>
     </row>
     <row r="4455" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4455" t="s">
-        <v>8554</v>
+        <v>8546</v>
       </c>
       <c r="B4455" t="s">
-        <v>8555</v>
+        <v>8547</v>
       </c>
     </row>
     <row r="4456" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4456" t="s">
-        <v>8556</v>
+        <v>8548</v>
       </c>
       <c r="B4456" t="s">
-        <v>8557</v>
+        <v>8549</v>
       </c>
     </row>
     <row r="4457" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4457" t="s">
-        <v>8558</v>
+        <v>8550</v>
       </c>
       <c r="B4457" t="s">
-        <v>8559</v>
+        <v>8551</v>
       </c>
     </row>
     <row r="4458" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4458" t="s">
-        <v>8560</v>
+        <v>8552</v>
       </c>
       <c r="B4458" t="s">
-        <v>8561</v>
+        <v>8553</v>
       </c>
     </row>
     <row r="4459" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4459" t="s">
-        <v>8562</v>
+        <v>8554</v>
       </c>
       <c r="B4459" t="s">
-        <v>8563</v>
+        <v>8555</v>
       </c>
     </row>
     <row r="4460" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4460" t="s">
-        <v>8564</v>
+        <v>8556</v>
       </c>
       <c r="B4460" t="s">
-        <v>8565</v>
+        <v>8557</v>
       </c>
     </row>
     <row r="4461" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4461" t="s">
-        <v>8566</v>
+        <v>8558</v>
       </c>
       <c r="B4461" t="s">
-        <v>8567</v>
+        <v>8559</v>
       </c>
     </row>
     <row r="4462" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4462" t="s">
-        <v>8568</v>
+        <v>8560</v>
       </c>
       <c r="B4462" t="s">
-        <v>8569</v>
+        <v>8561</v>
       </c>
     </row>
     <row r="4463" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4463" t="s">
-        <v>8570</v>
+        <v>8562</v>
       </c>
       <c r="B4463" t="s">
-        <v>8571</v>
+        <v>8563</v>
       </c>
     </row>
     <row r="4464" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4464" t="s">
-        <v>8572</v>
+        <v>8564</v>
       </c>
       <c r="B4464" t="s">
-        <v>8573</v>
+        <v>8565</v>
       </c>
     </row>
     <row r="4465" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4465" t="s">
-        <v>8574</v>
+        <v>8566</v>
       </c>
       <c r="B4465" t="s">
-        <v>8575</v>
+        <v>8567</v>
       </c>
     </row>
     <row r="4466" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4466" t="s">
-        <v>8576</v>
+        <v>8568</v>
       </c>
       <c r="B4466" t="s">
-        <v>8577</v>
+        <v>8569</v>
       </c>
     </row>
     <row r="4467" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4467" t="s">
-        <v>8578</v>
+        <v>8570</v>
       </c>
       <c r="B4467" t="s">
-        <v>8579</v>
+        <v>8571</v>
       </c>
     </row>
     <row r="4468" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4468" t="s">
-        <v>8580</v>
+        <v>8572</v>
       </c>
       <c r="B4468" t="s">
-        <v>8581</v>
+        <v>8573</v>
       </c>
     </row>
     <row r="4469" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4469" t="s">
-        <v>8582</v>
+        <v>8574</v>
       </c>
       <c r="B4469" t="s">
-        <v>8583</v>
+        <v>8575</v>
       </c>
     </row>
     <row r="4470" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4470" t="s">
-        <v>8584</v>
+        <v>8576</v>
       </c>
       <c r="B4470" t="s">
-        <v>8585</v>
+        <v>8577</v>
       </c>
     </row>
     <row r="4471" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4471" t="s">
-        <v>8586</v>
+        <v>8578</v>
       </c>
       <c r="B4471" t="s">
-        <v>8587</v>
+        <v>8579</v>
       </c>
     </row>
     <row r="4472" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4472" t="s">
-        <v>8588</v>
+        <v>8580</v>
       </c>
       <c r="B4472" t="s">
-        <v>8589</v>
+        <v>8581</v>
       </c>
     </row>
     <row r="4473" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4473" t="s">
-        <v>8590</v>
+        <v>8582</v>
       </c>
       <c r="B4473" t="s">
-        <v>8591</v>
+        <v>8583</v>
       </c>
     </row>
     <row r="4474" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4474" t="s">
-        <v>8592</v>
+        <v>8584</v>
       </c>
       <c r="B4474" t="s">
-        <v>8593</v>
+        <v>8585</v>
       </c>
     </row>
     <row r="4475" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4475" t="s">
-        <v>8594</v>
+        <v>8586</v>
       </c>
       <c r="B4475" t="s">
-        <v>8595</v>
+        <v>8587</v>
       </c>
     </row>
     <row r="4476" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4476" t="s">
-        <v>8596</v>
+        <v>8588</v>
       </c>
       <c r="B4476" t="s">
-        <v>8597</v>
+        <v>8589</v>
       </c>
     </row>
     <row r="4477" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4477" t="s">
-        <v>8598</v>
+        <v>8590</v>
       </c>
       <c r="B4477" t="s">
-        <v>8599</v>
+        <v>8591</v>
       </c>
     </row>
     <row r="4478" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4478" t="s">
-        <v>8600</v>
+        <v>8592</v>
       </c>
       <c r="B4478" t="s">
-        <v>8601</v>
+        <v>8593</v>
       </c>
     </row>
     <row r="4479" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4479" t="s">
-        <v>8602</v>
+        <v>8594</v>
       </c>
       <c r="B4479" t="s">
-        <v>8603</v>
+        <v>8595</v>
       </c>
     </row>
     <row r="4480" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4480" t="s">
-        <v>8604</v>
+        <v>8596</v>
       </c>
       <c r="B4480" t="s">
-        <v>8605</v>
+        <v>8597</v>
       </c>
     </row>
     <row r="4481" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4481" t="s">
-        <v>8606</v>
+        <v>8598</v>
       </c>
       <c r="B4481" t="s">
-        <v>8607</v>
+        <v>8599</v>
       </c>
     </row>
     <row r="4482" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4482" t="s">
-        <v>8608</v>
+        <v>8600</v>
       </c>
       <c r="B4482" t="s">
-        <v>8609</v>
+        <v>8601</v>
       </c>
     </row>
     <row r="4483" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4483" t="s">
-        <v>8610</v>
+        <v>8602</v>
       </c>
       <c r="B4483" t="s">
-        <v>8611</v>
+        <v>8603</v>
       </c>
     </row>
     <row r="4484" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4484" t="s">
-        <v>8612</v>
+        <v>8604</v>
       </c>
       <c r="B4484" t="s">
-        <v>8613</v>
+        <v>8605</v>
       </c>
     </row>
     <row r="4485" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4485" t="s">
-        <v>8614</v>
+        <v>8606</v>
       </c>
       <c r="B4485" t="s">
-        <v>8615</v>
+        <v>8607</v>
       </c>
     </row>
     <row r="4486" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4486" t="s">
-        <v>8616</v>
+        <v>8608</v>
       </c>
       <c r="B4486" t="s">
-        <v>8617</v>
+        <v>8609</v>
       </c>
     </row>
     <row r="4487" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4487" t="s">
-        <v>8618</v>
+        <v>8610</v>
       </c>
       <c r="B4487" t="s">
-        <v>8619</v>
+        <v>8611</v>
       </c>
     </row>
     <row r="4488" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4488" t="s">
-        <v>8620</v>
+        <v>8612</v>
       </c>
       <c r="B4488" t="s">
-        <v>8621</v>
+        <v>8613</v>
       </c>
     </row>
     <row r="4489" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4489" t="s">
-        <v>8622</v>
+        <v>8614</v>
       </c>
       <c r="B4489" t="s">
-        <v>8623</v>
+        <v>8615</v>
       </c>
     </row>
     <row r="4490" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4490" t="s">
-        <v>8624</v>
+        <v>8616</v>
       </c>
       <c r="B4490" t="s">
-        <v>8625</v>
+        <v>8617</v>
       </c>
     </row>
     <row r="4491" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4491" t="s">
-        <v>8626</v>
+        <v>8618</v>
       </c>
       <c r="B4491" t="s">
-        <v>8627</v>
+        <v>8619</v>
       </c>
     </row>
     <row r="4492" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4492" t="s">
-        <v>8628</v>
+        <v>8620</v>
       </c>
       <c r="B4492" t="s">
-        <v>8629</v>
+        <v>8621</v>
       </c>
     </row>
     <row r="4493" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4493" t="s">
-        <v>8630</v>
+        <v>8622</v>
       </c>
       <c r="B4493" t="s">
-        <v>8631</v>
+        <v>8623</v>
       </c>
     </row>
     <row r="4494" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4494" t="s">
-        <v>8632</v>
+        <v>8624</v>
       </c>
       <c r="B4494" t="s">
-        <v>8633</v>
+        <v>8625</v>
       </c>
     </row>
     <row r="4495" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4495" t="s">
-        <v>8634</v>
+        <v>8626</v>
       </c>
       <c r="B4495" t="s">
-        <v>8635</v>
+        <v>8627</v>
       </c>
     </row>
     <row r="4496" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4496" t="s">
-        <v>8636</v>
+        <v>8628</v>
       </c>
       <c r="B4496" t="s">
-        <v>8637</v>
+        <v>8629</v>
       </c>
     </row>
     <row r="4497" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4497" t="s">
-        <v>8638</v>
+        <v>8630</v>
       </c>
       <c r="B4497" t="s">
-        <v>8639</v>
+        <v>8631</v>
       </c>
     </row>
     <row r="4498" spans="1:2" x14ac:dyDescent="0.25">
@@ -63252,7 +63252,7 @@
         <v>5404</v>
       </c>
       <c r="B4498" t="s">
-        <v>8640</v>
+        <v>8632</v>
       </c>
     </row>
     <row r="4499" spans="1:2" x14ac:dyDescent="0.25">
@@ -63260,7 +63260,7 @@
         <v>5406</v>
       </c>
       <c r="B4499" t="s">
-        <v>8641</v>
+        <v>8633</v>
       </c>
     </row>
     <row r="4500" spans="1:2" x14ac:dyDescent="0.25">
@@ -63268,7 +63268,7 @@
         <v>5408</v>
       </c>
       <c r="B4500" t="s">
-        <v>8642</v>
+        <v>8634</v>
       </c>
     </row>
     <row r="4501" spans="1:2" x14ac:dyDescent="0.25">
@@ -63276,556 +63276,556 @@
         <v>5410</v>
       </c>
       <c r="B4501" t="s">
-        <v>8643</v>
+        <v>8635</v>
       </c>
     </row>
     <row r="4502" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4502" t="s">
-        <v>8644</v>
+        <v>8636</v>
       </c>
       <c r="B4502" t="s">
-        <v>8645</v>
+        <v>8637</v>
       </c>
     </row>
     <row r="4503" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4503" t="s">
-        <v>8646</v>
+        <v>8638</v>
       </c>
       <c r="B4503" t="s">
-        <v>8647</v>
+        <v>8639</v>
       </c>
     </row>
     <row r="4504" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4504" t="s">
-        <v>8648</v>
+        <v>8640</v>
       </c>
       <c r="B4504" t="s">
-        <v>8649</v>
+        <v>8641</v>
       </c>
     </row>
     <row r="4505" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4505" t="s">
-        <v>8650</v>
+        <v>8642</v>
       </c>
       <c r="B4505" t="s">
-        <v>8651</v>
+        <v>8643</v>
       </c>
     </row>
     <row r="4506" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4506" t="s">
-        <v>8652</v>
+        <v>8644</v>
       </c>
       <c r="B4506" t="s">
-        <v>8653</v>
+        <v>8645</v>
       </c>
     </row>
     <row r="4507" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4507" t="s">
-        <v>8654</v>
+        <v>8646</v>
       </c>
       <c r="B4507" t="s">
-        <v>8655</v>
+        <v>8647</v>
       </c>
     </row>
     <row r="4508" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4508" t="s">
-        <v>8656</v>
+        <v>8648</v>
       </c>
       <c r="B4508" t="s">
-        <v>8657</v>
+        <v>8649</v>
       </c>
     </row>
     <row r="4509" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4509" t="s">
-        <v>8658</v>
+        <v>8650</v>
       </c>
       <c r="B4509" t="s">
-        <v>8659</v>
+        <v>8651</v>
       </c>
     </row>
     <row r="4510" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4510" t="s">
-        <v>8660</v>
+        <v>8652</v>
       </c>
       <c r="B4510" t="s">
-        <v>8661</v>
+        <v>8653</v>
       </c>
     </row>
     <row r="4511" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4511" t="s">
-        <v>8662</v>
+        <v>8654</v>
       </c>
       <c r="B4511" t="s">
-        <v>8663</v>
+        <v>8655</v>
       </c>
     </row>
     <row r="4512" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4512" t="s">
-        <v>8664</v>
+        <v>8656</v>
       </c>
       <c r="B4512" t="s">
-        <v>8665</v>
+        <v>8657</v>
       </c>
     </row>
     <row r="4513" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4513" t="s">
-        <v>8666</v>
+        <v>8658</v>
       </c>
       <c r="B4513" t="s">
-        <v>8667</v>
+        <v>8659</v>
       </c>
     </row>
     <row r="4514" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4514" t="s">
-        <v>8668</v>
+        <v>8660</v>
       </c>
       <c r="B4514" t="s">
-        <v>8669</v>
+        <v>8661</v>
       </c>
     </row>
     <row r="4515" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4515" t="s">
-        <v>8670</v>
+        <v>8662</v>
       </c>
       <c r="B4515" t="s">
-        <v>8671</v>
+        <v>8663</v>
       </c>
     </row>
     <row r="4516" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4516" t="s">
-        <v>8672</v>
+        <v>8664</v>
       </c>
       <c r="B4516" t="s">
-        <v>8673</v>
+        <v>8665</v>
       </c>
     </row>
     <row r="4517" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4517" t="s">
-        <v>8674</v>
+        <v>8666</v>
       </c>
       <c r="B4517" t="s">
-        <v>8675</v>
+        <v>8667</v>
       </c>
     </row>
     <row r="4518" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4518" t="s">
-        <v>8676</v>
+        <v>8668</v>
       </c>
       <c r="B4518" t="s">
-        <v>8677</v>
+        <v>8669</v>
       </c>
     </row>
     <row r="4519" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4519" t="s">
-        <v>8678</v>
+        <v>8670</v>
       </c>
       <c r="B4519" t="s">
-        <v>8679</v>
+        <v>8671</v>
       </c>
     </row>
     <row r="4520" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4520" t="s">
-        <v>8680</v>
+        <v>8672</v>
       </c>
       <c r="B4520" t="s">
-        <v>8681</v>
+        <v>8673</v>
       </c>
     </row>
     <row r="4521" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4521" t="s">
-        <v>8682</v>
+        <v>8674</v>
       </c>
       <c r="B4521" t="s">
-        <v>8683</v>
+        <v>8675</v>
       </c>
     </row>
     <row r="4522" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4522" t="s">
-        <v>8684</v>
+        <v>8676</v>
       </c>
       <c r="B4522" t="s">
-        <v>8685</v>
+        <v>8677</v>
       </c>
     </row>
     <row r="4523" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4523" t="s">
-        <v>8686</v>
+        <v>8678</v>
       </c>
       <c r="B4523" t="s">
-        <v>8687</v>
+        <v>8679</v>
       </c>
     </row>
     <row r="4524" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4524" t="s">
-        <v>8688</v>
+        <v>8680</v>
       </c>
       <c r="B4524" t="s">
-        <v>8689</v>
+        <v>8681</v>
       </c>
     </row>
     <row r="4525" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4525" t="s">
-        <v>8690</v>
+        <v>8682</v>
       </c>
       <c r="B4525" t="s">
-        <v>8691</v>
+        <v>8683</v>
       </c>
     </row>
     <row r="4526" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4526" t="s">
-        <v>8692</v>
+        <v>8684</v>
       </c>
       <c r="B4526" t="s">
-        <v>8693</v>
+        <v>8685</v>
       </c>
     </row>
     <row r="4527" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4527" t="s">
-        <v>8694</v>
+        <v>8686</v>
       </c>
       <c r="B4527" t="s">
-        <v>8695</v>
+        <v>8687</v>
       </c>
     </row>
     <row r="4528" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4528" t="s">
-        <v>8696</v>
+        <v>8688</v>
       </c>
       <c r="B4528" t="s">
-        <v>8697</v>
+        <v>8689</v>
       </c>
     </row>
     <row r="4529" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4529" t="s">
-        <v>8698</v>
+        <v>8690</v>
       </c>
       <c r="B4529" t="s">
-        <v>8699</v>
+        <v>8691</v>
       </c>
     </row>
     <row r="4530" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4530" t="s">
-        <v>8700</v>
+        <v>8692</v>
       </c>
       <c r="B4530" t="s">
-        <v>8701</v>
+        <v>8693</v>
       </c>
     </row>
     <row r="4531" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4531" t="s">
-        <v>8702</v>
+        <v>8694</v>
       </c>
       <c r="B4531" t="s">
-        <v>8703</v>
+        <v>8695</v>
       </c>
     </row>
     <row r="4532" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4532" t="s">
-        <v>8704</v>
+        <v>8696</v>
       </c>
       <c r="B4532" t="s">
-        <v>8705</v>
+        <v>8697</v>
       </c>
     </row>
     <row r="4533" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4533" t="s">
-        <v>8706</v>
+        <v>8698</v>
       </c>
       <c r="B4533" t="s">
-        <v>8707</v>
+        <v>8699</v>
       </c>
     </row>
     <row r="4534" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4534" t="s">
-        <v>8708</v>
+        <v>8700</v>
       </c>
       <c r="B4534" t="s">
-        <v>8709</v>
+        <v>8701</v>
       </c>
     </row>
     <row r="4535" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4535" t="s">
-        <v>8710</v>
+        <v>8702</v>
       </c>
       <c r="B4535" t="s">
-        <v>8711</v>
+        <v>8703</v>
       </c>
     </row>
     <row r="4536" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4536" t="s">
-        <v>8712</v>
+        <v>8704</v>
       </c>
       <c r="B4536" t="s">
-        <v>8713</v>
+        <v>8705</v>
       </c>
     </row>
     <row r="4537" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4537" t="s">
-        <v>8714</v>
+        <v>8706</v>
       </c>
       <c r="B4537" t="s">
-        <v>8715</v>
+        <v>8707</v>
       </c>
     </row>
     <row r="4538" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4538" t="s">
-        <v>8716</v>
+        <v>8708</v>
       </c>
       <c r="B4538" t="s">
-        <v>8717</v>
+        <v>8709</v>
       </c>
     </row>
     <row r="4539" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4539" t="s">
-        <v>8718</v>
+        <v>8710</v>
       </c>
       <c r="B4539" t="s">
-        <v>8719</v>
+        <v>8711</v>
       </c>
     </row>
     <row r="4540" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4540" t="s">
-        <v>8720</v>
+        <v>8712</v>
       </c>
       <c r="B4540" t="s">
-        <v>8721</v>
+        <v>8713</v>
       </c>
     </row>
     <row r="4541" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4541" t="s">
-        <v>8722</v>
+        <v>8714</v>
       </c>
       <c r="B4541" t="s">
-        <v>8723</v>
+        <v>8715</v>
       </c>
     </row>
     <row r="4542" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4542" t="s">
-        <v>8724</v>
+        <v>8716</v>
       </c>
       <c r="B4542" t="s">
-        <v>8725</v>
+        <v>8717</v>
       </c>
     </row>
     <row r="4543" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4543" t="s">
-        <v>8726</v>
+        <v>8718</v>
       </c>
       <c r="B4543" t="s">
-        <v>8727</v>
+        <v>8719</v>
       </c>
     </row>
     <row r="4544" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4544" t="s">
-        <v>8728</v>
+        <v>8720</v>
       </c>
       <c r="B4544" t="s">
-        <v>8729</v>
+        <v>8721</v>
       </c>
     </row>
     <row r="4545" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4545" t="s">
-        <v>8730</v>
+        <v>8722</v>
       </c>
       <c r="B4545" t="s">
-        <v>8731</v>
+        <v>8723</v>
       </c>
     </row>
     <row r="4546" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4546" t="s">
-        <v>8732</v>
+        <v>8724</v>
       </c>
       <c r="B4546" t="s">
-        <v>8733</v>
+        <v>8725</v>
       </c>
     </row>
     <row r="4547" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4547" t="s">
-        <v>8734</v>
+        <v>8726</v>
       </c>
       <c r="B4547" t="s">
-        <v>8735</v>
+        <v>8727</v>
       </c>
     </row>
     <row r="4548" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4548" t="s">
-        <v>8736</v>
+        <v>8728</v>
       </c>
       <c r="B4548" t="s">
-        <v>8737</v>
+        <v>8729</v>
       </c>
     </row>
     <row r="4549" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4549" t="s">
-        <v>8738</v>
+        <v>8730</v>
       </c>
       <c r="B4549" t="s">
-        <v>8739</v>
+        <v>8731</v>
       </c>
     </row>
     <row r="4550" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4550" t="s">
-        <v>8740</v>
+        <v>8732</v>
       </c>
       <c r="B4550" t="s">
-        <v>8741</v>
+        <v>8733</v>
       </c>
     </row>
     <row r="4551" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4551" t="s">
-        <v>8742</v>
+        <v>8734</v>
       </c>
       <c r="B4551" t="s">
-        <v>8743</v>
+        <v>8735</v>
       </c>
     </row>
     <row r="4552" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4552" t="s">
-        <v>8744</v>
+        <v>8736</v>
       </c>
       <c r="B4552" t="s">
-        <v>8745</v>
+        <v>8737</v>
       </c>
     </row>
     <row r="4553" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4553" t="s">
-        <v>8746</v>
+        <v>8738</v>
       </c>
       <c r="B4553" t="s">
-        <v>8747</v>
+        <v>8739</v>
       </c>
     </row>
     <row r="4554" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4554" t="s">
-        <v>8748</v>
+        <v>8740</v>
       </c>
       <c r="B4554" t="s">
-        <v>8749</v>
+        <v>8741</v>
       </c>
     </row>
     <row r="4555" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4555" t="s">
-        <v>8750</v>
+        <v>8742</v>
       </c>
       <c r="B4555" t="s">
-        <v>8751</v>
+        <v>8743</v>
       </c>
     </row>
     <row r="4556" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4556" t="s">
-        <v>8752</v>
+        <v>8744</v>
       </c>
       <c r="B4556" t="s">
-        <v>8753</v>
+        <v>8745</v>
       </c>
     </row>
     <row r="4557" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4557" t="s">
-        <v>8754</v>
+        <v>8746</v>
       </c>
       <c r="B4557" t="s">
-        <v>8755</v>
+        <v>8747</v>
       </c>
     </row>
     <row r="4558" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4558" t="s">
-        <v>8756</v>
+        <v>8748</v>
       </c>
       <c r="B4558" t="s">
-        <v>8757</v>
+        <v>8749</v>
       </c>
     </row>
     <row r="4559" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4559" t="s">
-        <v>8758</v>
+        <v>8750</v>
       </c>
       <c r="B4559" t="s">
-        <v>8759</v>
+        <v>8751</v>
       </c>
     </row>
     <row r="4560" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4560" t="s">
-        <v>8760</v>
+        <v>8752</v>
       </c>
       <c r="B4560" t="s">
-        <v>8761</v>
+        <v>8753</v>
       </c>
     </row>
     <row r="4561" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4561" t="s">
-        <v>8762</v>
+        <v>8754</v>
       </c>
       <c r="B4561" t="s">
-        <v>8763</v>
+        <v>8755</v>
       </c>
     </row>
     <row r="4562" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4562" t="s">
-        <v>8764</v>
+        <v>8756</v>
       </c>
       <c r="B4562" t="s">
-        <v>8765</v>
+        <v>8757</v>
       </c>
     </row>
     <row r="4563" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4563" t="s">
-        <v>8766</v>
+        <v>8758</v>
       </c>
       <c r="B4563" t="s">
-        <v>8767</v>
+        <v>8759</v>
       </c>
     </row>
     <row r="4564" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4564" t="s">
-        <v>8768</v>
+        <v>8760</v>
       </c>
       <c r="B4564" t="s">
-        <v>8769</v>
+        <v>8761</v>
       </c>
     </row>
     <row r="4565" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4565" t="s">
-        <v>8770</v>
+        <v>8762</v>
       </c>
       <c r="B4565" t="s">
-        <v>8771</v>
+        <v>8763</v>
       </c>
     </row>
     <row r="4566" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4566" t="s">
-        <v>8772</v>
+        <v>8764</v>
       </c>
       <c r="B4566" t="s">
-        <v>8773</v>
+        <v>8765</v>
       </c>
     </row>
     <row r="4567" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4567" t="s">
-        <v>8774</v>
+        <v>8766</v>
       </c>
       <c r="B4567" t="s">
-        <v>8775</v>
+        <v>8767</v>
       </c>
     </row>
     <row r="4568" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4568" t="s">
-        <v>8776</v>
+        <v>8768</v>
       </c>
       <c r="B4568" t="s">
-        <v>8777</v>
+        <v>8769</v>
       </c>
     </row>
     <row r="4569" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4569" t="s">
-        <v>8778</v>
+        <v>8770</v>
       </c>
       <c r="B4569" t="s">
-        <v>8779</v>
+        <v>8771</v>
       </c>
     </row>
     <row r="4570" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4570" t="s">
-        <v>8785</v>
+        <v>8777</v>
       </c>
       <c r="B4570" t="s">
         <v>979</v>
@@ -63833,7 +63833,7 @@
     </row>
     <row r="4571" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4571" t="s">
-        <v>8786</v>
+        <v>8778</v>
       </c>
       <c r="B4571" t="s">
         <v>981</v>
@@ -63841,7 +63841,7 @@
     </row>
     <row r="4572" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4572" t="s">
-        <v>8787</v>
+        <v>8779</v>
       </c>
       <c r="B4572" t="s">
         <v>983</v>
@@ -63849,14 +63849,13 @@
     </row>
     <row r="4573" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4573" t="s">
-        <v>8785</v>
+        <v>8777</v>
       </c>
       <c r="B4573" t="s">
         <v>985</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B4573" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>